<commit_message>
Apply r/financialmodelling feedback: blended betas, implied discount rate, WACC x terminal growth grid
Betas now use 0.67 x regression + 0.33 in the calculator and the four example workbooks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/Amazon DCF.xlsx
+++ b/examples/Amazon DCF.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207C8025-0261-8B4F-ABCB-DE8CA2D61E85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12BAE78A-6C1D-654F-949E-C3FC56729EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="34200" windowHeight="19220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="34200" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DCF" sheetId="1" r:id="rId1"/>
@@ -84,9 +84,6 @@
     <t>Beta</t>
   </si>
   <si>
-    <t>Judgment. 5-year monthly regression against the S&amp;P 500 gives 1.50, pushed up by the 2022 fall. 1.3 is typical for large internet companies</t>
-  </si>
-  <si>
     <t>Equity risk premium</t>
   </si>
   <si>
@@ -313,6 +310,9 @@
   </si>
   <si>
     <t>Sources: Amazon FY2025 Form 10-K and 2026 10-Q filings via SEC EDGAR; analyst estimates and price from Yahoo Finance, 14 Oct 2026.</t>
+  </si>
+  <si>
+    <t>Judgment. 5-year monthly regression against the S&amp;P 500 gives 1.50, pushed up by the 2022 fall. Blended toward 1: 0.67 × 1.50 + 0.33 = 1.34</t>
   </si>
 </sst>
 </file>
@@ -321,12 +321,12 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.0%;\(0.0%\);&quot;-&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
-    <numFmt numFmtId="170" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);&quot;-&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -390,27 +390,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -822,204 +822,204 @@
         <v>17</v>
       </c>
       <c r="C13" s="6">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="P13" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14" s="7">
         <v>4.4999999999999998E-2</v>
       </c>
       <c r="P14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" s="5">
         <v>0</v>
       </c>
       <c r="P15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="8">
         <f>C12+C13*C14+C15</f>
-        <v>0.1104</v>
+        <v>0.11219999999999999</v>
       </c>
       <c r="P16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" s="5">
         <v>5.7000000000000002E-2</v>
       </c>
       <c r="P17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C18" s="5">
         <v>0.21</v>
       </c>
       <c r="P18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19" s="9">
         <f>C11/(C11+C7*C8)</f>
         <v>4.6026062736998857E-2</v>
       </c>
       <c r="P19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" s="10">
         <f>C16*(1-C19)+C17*(1-C18)*C19</f>
-        <v>0.10739127627888238</v>
+        <v>0.10910842936595579</v>
       </c>
       <c r="P20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C21" s="5">
         <v>0.18</v>
       </c>
       <c r="P21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C22" s="6">
         <v>1.2</v>
       </c>
       <c r="P22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" s="5">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="P23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24" s="5">
         <v>0.15</v>
       </c>
       <c r="P24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" s="7">
         <v>0.17</v>
       </c>
       <c r="P25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C26" s="5">
         <v>0.18</v>
       </c>
       <c r="P26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.2">
       <c r="D30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="E30" s="11" t="s">
+      <c r="F30" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F30" s="11" t="s">
+      <c r="G30" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="H30" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="H30" s="11" t="s">
+      <c r="I30" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="I30" s="11" t="s">
+      <c r="J30" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="J30" s="11" t="s">
+      <c r="K30" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="K30" s="11" t="s">
+      <c r="L30" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="L30" s="11" t="s">
+      <c r="M30" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="M30" s="11" t="s">
+      <c r="N30" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="N30" s="11" t="s">
+      <c r="O30" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="O30" s="11" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E31" s="7">
         <v>0.156</v>
@@ -1056,12 +1056,12 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="P31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B32" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D32" s="12">
         <f>C9</f>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D33" s="9">
         <f>79975/716924</f>
@@ -1155,12 +1155,12 @@
         <v>0.17</v>
       </c>
       <c r="P33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E34" s="12">
         <f t="shared" ref="E34:O34" si="1">E32*E33</f>
@@ -1209,7 +1209,7 @@
     </row>
     <row r="35" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E35" s="12">
         <f t="shared" ref="E35:N35" si="2">E34*(1-$C$21)</f>
@@ -1258,7 +1258,7 @@
     </row>
     <row r="36" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E36" s="12">
         <f t="shared" ref="E36:N36" si="3">-MAX(0,E32-D32)/$C$22</f>
@@ -1305,12 +1305,12 @@
         <v>-43324.614873318496</v>
       </c>
       <c r="P36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E37" s="13">
         <f t="shared" ref="E37:O37" si="4">E35+E36</f>
@@ -1359,7 +1359,7 @@
     </row>
     <row r="38" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E38" s="9">
         <f>(DATE(2026,12,31)-$C$6)/365</f>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E39" s="14">
         <f>E38/2</f>
@@ -1440,147 +1440,147 @@
     </row>
     <row r="40" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E40" s="15">
         <f t="shared" ref="E40:N40" si="5">1/(1+$C$20)^E39</f>
-        <v>0.9891597998815379</v>
+        <v>0.98899605276136837</v>
       </c>
       <c r="F40" s="15">
         <f t="shared" si="5"/>
-        <v>0.92978463937241551</v>
+        <v>0.9287570288440562</v>
       </c>
       <c r="G40" s="15">
         <f t="shared" si="5"/>
-        <v>0.83961708863801909</v>
+        <v>0.83739065023155479</v>
       </c>
       <c r="H40" s="15">
         <f t="shared" si="5"/>
-        <v>0.75819369957414418</v>
+        <v>0.75501242985797701</v>
       </c>
       <c r="I40" s="15">
         <f t="shared" si="5"/>
-        <v>0.68466649125309043</v>
+        <v>0.68073815856723319</v>
       </c>
       <c r="J40" s="15">
         <f t="shared" si="5"/>
-        <v>0.61826971723467494</v>
+        <v>0.61377061118937737</v>
       </c>
       <c r="K40" s="15">
         <f t="shared" si="5"/>
-        <v>0.55831189072774634</v>
+        <v>0.55339098949978383</v>
       </c>
       <c r="L40" s="15">
         <f t="shared" si="5"/>
-        <v>0.50416858312611679</v>
+        <v>0.49895120697634671</v>
       </c>
       <c r="M40" s="15">
         <f t="shared" si="5"/>
-        <v>0.45527592091952535</v>
+        <v>0.44986693254290938</v>
       </c>
       <c r="N40" s="15">
         <f t="shared" si="5"/>
-        <v>0.41112471325344802</v>
+        <v>0.4056113186337289</v>
       </c>
     </row>
     <row r="41" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B41" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E41" s="13">
         <f t="shared" ref="E41:N41" si="6">E37*E38*E40</f>
-        <v>-307.7573758476974</v>
+        <v>-307.70642919174554</v>
       </c>
       <c r="F41" s="13">
         <f t="shared" si="6"/>
-        <v>11795.276646423974</v>
+        <v>11782.240347529041</v>
       </c>
       <c r="G41" s="13">
         <f t="shared" si="6"/>
-        <v>33743.617003030937</v>
+        <v>33654.138018044534</v>
       </c>
       <c r="H41" s="13">
         <f t="shared" si="6"/>
-        <v>43486.003635047091</v>
+        <v>43303.542732880516</v>
       </c>
       <c r="I41" s="13">
         <f t="shared" si="6"/>
-        <v>56545.222086476417</v>
+        <v>56220.789027477404</v>
       </c>
       <c r="J41" s="13">
         <f t="shared" si="6"/>
-        <v>61735.383468667133</v>
+        <v>61286.139345544056</v>
       </c>
       <c r="K41" s="13">
         <f t="shared" si="6"/>
-        <v>66245.981129834341</v>
+        <v>65662.096144930183</v>
       </c>
       <c r="L41" s="13">
         <f t="shared" si="6"/>
-        <v>69951.973616371179</v>
+        <v>69228.077342405799</v>
       </c>
       <c r="M41" s="13">
         <f t="shared" si="6"/>
-        <v>72754.155101825803</v>
+        <v>71889.786130803841</v>
       </c>
       <c r="N41" s="13">
         <f t="shared" si="6"/>
-        <v>74583.732682801477</v>
+        <v>73583.526328778607</v>
       </c>
     </row>
     <row r="43" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B43" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D44" s="12">
         <f>SUM(E41:N41)</f>
-        <v>490533.58799463062</v>
+        <v>486302.6289892022</v>
       </c>
     </row>
     <row r="45" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D45" s="12">
         <f>O37/(C20-C23)</f>
-        <v>2629199.1597915674</v>
+        <v>2575521.5737541057</v>
       </c>
     </row>
     <row r="46" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" s="12">
         <f>D45/(1+C20)^(E38+9)</f>
-        <v>1027179.9164710104</v>
+        <v>991946.51193962269</v>
       </c>
     </row>
     <row r="47" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D47" s="13">
         <f>D44+D46</f>
-        <v>1517713.504465641</v>
+        <v>1478249.1409288249</v>
       </c>
     </row>
     <row r="48" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D48" s="9">
         <f>D46/D47</f>
-        <v>0.67679434455099063</v>
+        <v>0.67102796441765911</v>
       </c>
     </row>
     <row r="49" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D49" s="12">
         <f>C10</f>
@@ -1589,25 +1589,25 @@
     </row>
     <row r="50" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B50" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D50" s="13">
         <f>D47+D49</f>
-        <v>1508477.504465641</v>
+        <v>1469013.1409288249</v>
       </c>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B51" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D51" s="20">
         <f>D50/C8</f>
-        <v>139.85124690261173</v>
+        <v>136.19249797695457</v>
       </c>
     </row>
     <row r="52" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D52" s="21">
         <f>C7</f>
@@ -1616,42 +1616,42 @@
     </row>
     <row r="53" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B53" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D53" s="16">
         <f>D51/D52-1</f>
-        <v>-0.44957790104450679</v>
+        <v>-0.46397788894460579</v>
       </c>
     </row>
     <row r="54" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" s="17">
         <f>C7/12.43</f>
         <v>20.440868865647627</v>
       </c>
       <c r="P54" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="55" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D55" s="17">
         <f>D51/12.43</f>
-        <v>11.25110594550376</v>
+        <v>10.956757681170924</v>
       </c>
     </row>
     <row r="58" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B58" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="59" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D59" s="18">
         <v>0.12</v>
@@ -1672,164 +1672,164 @@
     <row r="60" spans="2:16" x14ac:dyDescent="0.2">
       <c r="C60" s="18">
         <f>$C$20+(-0.03)</f>
-        <v>7.7391276278882384E-2</v>
+        <v>7.9108429365955787E-2</v>
       </c>
       <c r="D60" s="21">
         <f t="shared" ref="D60:H64" si="7">(SUMPRODUCT($E$37:$H$37,$E$38:$H$38,1/(1+$C60)^$E$39:$H$39)+SUMPRODUCT($I$32:$N$32*($I$33:$N$33+D$59-$C$25)*(1-$C$21)+$I$36:$N$36,1/(1+$C60)^$I$39:$N$39)+$O$32*D$59*(1-$C$26)*(1-$C$23/$C$24)/($C60-$C$23)/(1+$C60)^($E$38+9)+$C$10)/$C$8</f>
-        <v>166.0291984248114</v>
+        <v>159.52511293978012</v>
       </c>
       <c r="E60" s="21">
         <f t="shared" si="7"/>
-        <v>205.59474983178328</v>
+        <v>197.68053672648466</v>
       </c>
       <c r="F60" s="21">
         <f t="shared" si="7"/>
-        <v>245.16030123875527</v>
+        <v>235.83596051318929</v>
       </c>
       <c r="G60" s="21">
         <f t="shared" si="7"/>
-        <v>284.72585264572717</v>
+        <v>273.99138429989381</v>
       </c>
       <c r="H60" s="21">
         <f t="shared" si="7"/>
-        <v>324.29140405269908</v>
+        <v>312.14680808659836</v>
       </c>
       <c r="P60" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="61" spans="2:16" x14ac:dyDescent="0.2">
       <c r="C61" s="18">
         <f>$C$20+(-0.015)</f>
-        <v>9.2391276278882384E-2</v>
+        <v>9.4108429365955787E-2</v>
       </c>
       <c r="D61" s="21">
         <f t="shared" si="7"/>
-        <v>120.86953881405444</v>
+        <v>117.01156821836489</v>
       </c>
       <c r="E61" s="21">
         <f t="shared" si="7"/>
-        <v>150.56750708895694</v>
+        <v>145.85626591241123</v>
       </c>
       <c r="F61" s="21">
         <f t="shared" si="7"/>
-        <v>180.26547536385948</v>
+        <v>174.70096360645761</v>
       </c>
       <c r="G61" s="21">
         <f t="shared" si="7"/>
-        <v>209.96344363876199</v>
+        <v>203.54566130050395</v>
       </c>
       <c r="H61" s="21">
         <f t="shared" si="7"/>
-        <v>239.66141191366449</v>
+        <v>232.39035899455035</v>
       </c>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.2">
       <c r="C62" s="18">
         <f>$C$20+(0)</f>
-        <v>0.10739127627888238</v>
+        <v>0.10910842936595579</v>
       </c>
       <c r="D62" s="21">
         <f t="shared" si="7"/>
-        <v>92.925025415495242</v>
+        <v>90.405318908420881</v>
       </c>
       <c r="E62" s="21">
         <f t="shared" si="7"/>
-        <v>116.38813615905347</v>
+        <v>113.29890844268772</v>
       </c>
       <c r="F62" s="21">
         <f t="shared" si="7"/>
-        <v>139.85124690261173</v>
+        <v>136.19249797695457</v>
       </c>
       <c r="G62" s="21">
         <f t="shared" si="7"/>
-        <v>163.31435764617001</v>
+        <v>159.08608751122139</v>
       </c>
       <c r="H62" s="21">
         <f t="shared" si="7"/>
-        <v>186.77746838972826</v>
+        <v>181.97967704548819</v>
       </c>
     </row>
     <row r="63" spans="2:16" x14ac:dyDescent="0.2">
       <c r="C63" s="18">
         <f>$C$20+(0.015)</f>
-        <v>0.12239127627888238</v>
+        <v>0.12410842936595579</v>
       </c>
       <c r="D63" s="21">
         <f t="shared" si="7"/>
-        <v>74.153058164783857</v>
+        <v>72.39853903031603</v>
       </c>
       <c r="E63" s="21">
         <f t="shared" si="7"/>
-        <v>93.333240532027887</v>
+        <v>91.173001526710195</v>
       </c>
       <c r="F63" s="21">
         <f t="shared" si="7"/>
-        <v>112.51342289927196</v>
+        <v>109.94746402310442</v>
       </c>
       <c r="G63" s="21">
         <f t="shared" si="7"/>
-        <v>131.69360526651599</v>
+        <v>128.7219265194986</v>
       </c>
       <c r="H63" s="21">
         <f t="shared" si="7"/>
-        <v>150.87378763376003</v>
+        <v>147.49638901589276</v>
       </c>
     </row>
     <row r="64" spans="2:16" x14ac:dyDescent="0.2">
       <c r="C64" s="18">
         <f>$C$20+(0.03)</f>
-        <v>0.13739127627888237</v>
+        <v>0.1391084293659558</v>
       </c>
       <c r="D64" s="21">
         <f t="shared" si="7"/>
-        <v>60.81598386229556</v>
+        <v>59.536984956383577</v>
       </c>
       <c r="E64" s="21">
         <f t="shared" si="7"/>
-        <v>76.881902263508564</v>
+        <v>75.300150640521437</v>
       </c>
       <c r="F64" s="21">
         <f t="shared" si="7"/>
-        <v>92.947820664721604</v>
+        <v>91.063316324659326</v>
       </c>
       <c r="G64" s="21">
         <f t="shared" si="7"/>
-        <v>109.01373906593463</v>
+        <v>106.82648200879717</v>
       </c>
       <c r="H64" s="21">
         <f t="shared" si="7"/>
-        <v>125.07965746714763</v>
+        <v>122.58964769293507</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B66" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>